<commit_message>
Plan de pruebas final: 306 casos con resultados reales
</commit_message>
<xml_diff>
--- a/software_tienda_f/docs/Plan_de_Pruebas.xlsx
+++ b/software_tienda_f/docs/Plan_de_Pruebas.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Requisitos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan de pruebas'!$A$1:$H$306</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan de pruebas'!$A$1:$H$307</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requisitos'!$A$1:$D$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H306"/>
+  <dimension ref="A1:H307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4077,7 +4077,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Fecha 25/10/2026 06:09 visible: True</t>
+          <t>Fecha 25/10/2026 07:31 visible: True</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>Revisada por: prenomina-auxiliar (ID: 167 - Identificacion: None - Estado: ACTIVO); fecha: 2026-10-25 10:58:50.170151+00:00</t>
+          <t>Revisada por: prenomina-auxiliar (ID: 169 - Identificacion: None - Estado: ACTIVO); fecha: 2026-10-25 12:21:55.350990+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -6891,7 +6891,7 @@
       </c>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>Fecha respuesta: 2026-10-25 11:10:24.661817+00:00; respondida por: auxiliar-resp (ID: 1134 - Identificacion: None - Estado: ACTIVO)</t>
+          <t>Fecha respuesta: 2026-10-25 12:31:53.718454+00:00; respondida por: auxiliar-resp (ID: 1136 - Identificacion: None - Estado: ACTIVO)</t>
         </is>
       </c>
       <c r="G153" s="3" t="inlineStr">
@@ -9517,32 +9517,32 @@
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>RF-011</t>
+          <t>RF-010</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>Validar que tras cambiar la contraseña la sesión siga abierta.</t>
+          <t>Validar que un correo inicie sesión en su propia cuenta aunque otro usuario tenga ese texto como nombre de usuario.</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>actual: 'ClaveSegura1'; nueva: 'NuevaClave2'</t>
+          <t>Usuario A con username 'login-t61@example.com' y clave 'OtraClave9'; usuario B con ese correo; se ingresa el correo con la clave de B</t>
         </is>
       </c>
       <c r="E216" s="2" t="inlineStr">
         <is>
-          <t>Redirección al perfil y el perfil responde HTTP 200</t>
+          <t>Inicia sesión el usuario B (dueño del correo)</t>
         </is>
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>Redirección a /perfil/; perfil HTTP 200</t>
+          <t>Sesión iniciada para: login-t61</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: CambioContrasenaT61Test.test_cambio_valido_conserva_sesion</t>
+          <t>Prueba automatizada: LoginT61Test.test_login_correo_no_confunde_con_username</t>
         </is>
       </c>
       <c r="H216" s="2" t="inlineStr">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>Validar que el cambio de contraseña guarde la nueva clave.</t>
+          <t>Validar que tras cambiar la contraseña la sesión siga abierta.</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -9574,17 +9574,17 @@
       </c>
       <c r="E217" s="3" t="inlineStr">
         <is>
-          <t>La nueva contraseña queda activa</t>
+          <t>Redirección al perfil y el perfil responde HTTP 200</t>
         </is>
       </c>
       <c r="F217" s="3" t="inlineStr">
         <is>
-          <t>Nueva contraseña activa: True</t>
+          <t>Redirección a /perfil/; perfil HTTP 200</t>
         </is>
       </c>
       <c r="G217" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: CambioContrasenaT61Test.test_cambio_valido_guarda_clave</t>
+          <t>Prueba automatizada: CambioContrasenaT61Test.test_cambio_valido_conserva_sesion</t>
         </is>
       </c>
       <c r="H217" s="3" t="inlineStr">
@@ -9606,27 +9606,27 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Validar el mensaje cuando la contraseña actual es incorrecta.</t>
+          <t>Validar que el cambio de contraseña guarde la nueva clave.</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>actual: 'Incorrecta1'; nueva: 'NuevaClave2'</t>
+          <t>actual: 'ClaveSegura1'; nueva: 'NuevaClave2'</t>
         </is>
       </c>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>Tu contraseña actual es incorrecta.</t>
+          <t>La nueva contraseña queda activa</t>
         </is>
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; mensaje visible: True</t>
+          <t>Nueva contraseña activa: True</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: CambioContrasenaT61Test.test_contrasena_actual_incorrecta_muestra_error</t>
+          <t>Prueba automatizada: CambioContrasenaT61Test.test_cambio_valido_guarda_clave</t>
         </is>
       </c>
       <c r="H218" s="2" t="inlineStr">
@@ -9643,32 +9643,32 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>RF-012</t>
+          <t>RF-011</t>
         </is>
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Validar que perfil enmascare número de cuenta.</t>
+          <t>Validar el mensaje cuando la contraseña actual es incorrecta.</t>
         </is>
       </c>
       <c r="D219" s="3" t="inlineStr">
         <is>
-          <t>GET /perfil/ con cuenta '12345678'</t>
+          <t>actual: 'Incorrecta1'; nueva: 'NuevaClave2'</t>
         </is>
       </c>
       <c r="E219" s="3" t="inlineStr">
         <is>
-          <t>La respuesta muestra ****5678.</t>
+          <t>Tu contraseña actual es incorrecta.</t>
         </is>
       </c>
       <c r="F219" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200; texto: ****5678</t>
+          <t>HTTP 200; mensaje visible: True</t>
         </is>
       </c>
       <c r="G219" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: PagoEmpleadoTest.test_perfil_enmascara_cuenta</t>
+          <t>Prueba automatizada: CambioContrasenaT61Test.test_contrasena_actual_incorrecta_muestra_error</t>
         </is>
       </c>
       <c r="H219" s="3" t="inlineStr">
@@ -9690,27 +9690,27 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Validar que perfil muestre método de pago.</t>
+          <t>Validar que perfil enmascare número de cuenta.</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>GET /perfil/ como empleado con transferencia</t>
+          <t>GET /perfil/ con cuenta '12345678'</t>
         </is>
       </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t>La respuesta muestra Transferencia bancaria.</t>
+          <t>La respuesta muestra ****5678.</t>
         </is>
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; texto: Transferencia bancaria</t>
+          <t>HTTP 200; texto: ****5678</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: PagoEmpleadoTest.test_perfil_muestra_metodo_pago</t>
+          <t>Prueba automatizada: PagoEmpleadoTest.test_perfil_enmascara_cuenta</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
@@ -9732,27 +9732,27 @@
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Validar que perfil no exponga la cuenta completa.</t>
+          <t>Validar que perfil muestre método de pago.</t>
         </is>
       </c>
       <c r="D221" s="3" t="inlineStr">
         <is>
-          <t>GET /perfil/ con cuenta '12345678'</t>
+          <t>GET /perfil/ como empleado con transferencia</t>
         </is>
       </c>
       <c r="E221" s="3" t="inlineStr">
         <is>
-          <t>La respuesta no contiene 12345678.</t>
+          <t>La respuesta muestra Transferencia bancaria.</t>
         </is>
       </c>
       <c r="F221" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200; cuenta completa presente: False</t>
+          <t>HTTP 200; texto: Transferencia bancaria</t>
         </is>
       </c>
       <c r="G221" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: PagoEmpleadoTest.test_perfil_no_muestra_cuenta_completa</t>
+          <t>Prueba automatizada: PagoEmpleadoTest.test_perfil_muestra_metodo_pago</t>
         </is>
       </c>
       <c r="H221" s="3" t="inlineStr">
@@ -9774,27 +9774,27 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>Validar que el perfil no acepte un correo de otro usuario.</t>
+          <t>Validar que perfil no exponga la cuenta completa.</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>correo de otro usuario registrado</t>
+          <t>GET /perfil/ con cuenta '12345678'</t>
         </is>
       </c>
       <c r="E222" s="2" t="inlineStr">
         <is>
-          <t>Ya existe un usuario con ese correo electrónico.</t>
+          <t>La respuesta no contiene 12345678.</t>
         </is>
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; mensaje visible: True</t>
+          <t>HTTP 200; cuenta completa presente: False</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: PerfilPropioT61Test.test_correo_duplicado_muestra_mensaje</t>
+          <t>Prueba automatizada: PagoEmpleadoTest.test_perfil_no_muestra_cuenta_completa</t>
         </is>
       </c>
       <c r="H222" s="2" t="inlineStr">
@@ -9816,27 +9816,27 @@
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Validar que el empleado no pueda editar datos administrativos desde su perfil.</t>
+          <t>Validar que el perfil no acepte un correo de otro usuario.</t>
         </is>
       </c>
       <c r="D223" s="3" t="inlineStr">
         <is>
-          <t>Formulario de perfil propio</t>
+          <t>correo de otro usuario registrado</t>
         </is>
       </c>
       <c r="E223" s="3" t="inlineStr">
         <is>
-          <t>Sin campos salario_base, groups, identificacion ni estado</t>
+          <t>Ya existe un usuario con ese correo electrónico.</t>
         </is>
       </c>
       <c r="F223" s="3" t="inlineStr">
         <is>
-          <t>Campos del formulario: ['first_name', 'last_name', 'email']; administrativos expuestos: ninguno</t>
+          <t>HTTP 200; mensaje visible: True</t>
         </is>
       </c>
       <c r="G223" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: PerfilPropioT61Test.test_formulario_no_expone_campos_administrativos</t>
+          <t>Prueba automatizada: PerfilPropioT61Test.test_correo_duplicado_muestra_mensaje</t>
         </is>
       </c>
       <c r="H223" s="3" t="inlineStr">
@@ -9858,27 +9858,27 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>Validar que el perfil no acepte nombres con números.</t>
+          <t>Validar que el empleado no pueda editar datos administrativos desde su perfil.</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>nombres: 'Nombre2'</t>
+          <t>Formulario de perfil propio</t>
         </is>
       </c>
       <c r="E224" s="2" t="inlineStr">
         <is>
-          <t>El campo nombres solo puede contener letras y espacios.</t>
+          <t>Sin campos salario_base, groups, identificacion ni estado</t>
         </is>
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; mensaje visible: True</t>
+          <t>Campos del formulario: ['first_name', 'last_name', 'email']; administrativos expuestos: ninguno</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: PerfilPropioT61Test.test_nombre_con_numeros_muestra_mensaje</t>
+          <t>Prueba automatizada: PerfilPropioT61Test.test_formulario_no_expone_campos_administrativos</t>
         </is>
       </c>
       <c r="H224" s="2" t="inlineStr">
@@ -9900,27 +9900,27 @@
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Validar que el empleado actualice su correo.</t>
+          <t>Validar que el perfil no acepte nombres con números.</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
         <is>
-          <t>correo: 'nuevo-perfil@example.com'</t>
+          <t>nombres: 'Nombre2'</t>
         </is>
       </c>
       <c r="E225" s="3" t="inlineStr">
         <is>
-          <t>Correo guardado 'nuevo-perfil@example.com'</t>
+          <t>El campo nombres solo puede contener letras y espacios.</t>
         </is>
       </c>
       <c r="F225" s="3" t="inlineStr">
         <is>
-          <t>Correo guardado: nuevo-perfil@example.com</t>
+          <t>HTTP 200; mensaje visible: True</t>
         </is>
       </c>
       <c r="G225" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: PerfilPropioT61Test.test_vendedor_actualiza_correo</t>
+          <t>Prueba automatizada: PerfilPropioT61Test.test_nombre_con_numeros_muestra_mensaje</t>
         </is>
       </c>
       <c r="H225" s="3" t="inlineStr">
@@ -9942,27 +9942,27 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>Validar que el empleado actualice sus nombres y apellidos.</t>
+          <t>Validar que el empleado actualice su correo.</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>nombres: 'Nombre Nuevo'; apellidos: 'Apellido Nuevo'</t>
+          <t>correo: 'nuevo-perfil@example.com'</t>
         </is>
       </c>
       <c r="E226" s="2" t="inlineStr">
         <is>
-          <t>Perfil guardado con 'Nombre Nuevo Apellido Nuevo'</t>
+          <t>Correo guardado 'nuevo-perfil@example.com'</t>
         </is>
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>Nombre guardado: Nombre Nuevo Apellido Nuevo</t>
+          <t>Correo guardado: nuevo-perfil@example.com</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: PerfilPropioT61Test.test_vendedor_actualiza_nombres</t>
+          <t>Prueba automatizada: PerfilPropioT61Test.test_vendedor_actualiza_correo</t>
         </is>
       </c>
       <c r="H226" s="2" t="inlineStr">
@@ -9984,27 +9984,27 @@
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Validar edición que conserva identificación y correo propios.</t>
+          <t>Validar que el empleado actualice sus nombres y apellidos.</t>
         </is>
       </c>
       <c r="D227" s="3" t="inlineStr">
         <is>
-          <t>correo: 'EDITAR@example.com'; identificación: '9160616'</t>
+          <t>nombres: 'Nombre Nuevo'; apellidos: 'Apellido Nuevo'</t>
         </is>
       </c>
       <c r="E227" s="3" t="inlineStr">
         <is>
-          <t>El formulario de edición acepta los datos propios sin duplicidad.</t>
+          <t>Perfil guardado con 'Nombre Nuevo Apellido Nuevo'</t>
         </is>
       </c>
       <c r="F227" s="3" t="inlineStr">
         <is>
-          <t>Formulario válido: True</t>
+          <t>Nombre guardado: Nombre Nuevo Apellido Nuevo</t>
         </is>
       </c>
       <c r="G227" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ValidacionesGestionUsuarioTest.test_edicion_conserva_identificacion_y_correo</t>
+          <t>Prueba automatizada: PerfilPropioT61Test.test_vendedor_actualiza_nombres</t>
         </is>
       </c>
       <c r="H227" s="3" t="inlineStr">
@@ -10026,27 +10026,27 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>Integración: tras la aprobación el empleado ve su nómina y su último pago.</t>
+          <t>Validar edición que conserva identificación y correo propios.</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>Ciclo completo aprobado; el empleado consulta nómina y perfil</t>
+          <t>correo: 'EDITAR@example.com'; identificación: '9160616'</t>
         </is>
       </c>
       <c r="E228" s="2" t="inlineStr">
         <is>
-          <t>Consulta con montos ('$') y perfil con 'Último pago'</t>
+          <t>El formulario de edición acepta los datos propios sin duplicidad.</t>
         </is>
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>Montos en la consulta: True; 'Último pago' en el perfil: True</t>
+          <t>Formulario válido: True</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: IntegracionNominaTest.test_ciclo_completo_empleado_ve_pago</t>
+          <t>Prueba automatizada: ValidacionesGestionUsuarioTest.test_edicion_conserva_identificacion_y_correo</t>
         </is>
       </c>
       <c r="H228" s="2" t="inlineStr">
@@ -10068,27 +10068,27 @@
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Validar que el perfil del empleado muestre su último pago.</t>
+          <t>Integración: tras la aprobación el empleado ve su nómina y su último pago.</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
         <is>
-          <t>Pre-nómina aprobada; el empleado abre su perfil</t>
+          <t>Ciclo completo aprobado; el empleado consulta nómina y perfil</t>
         </is>
       </c>
       <c r="E229" s="3" t="inlineStr">
         <is>
-          <t>El perfil muestra 'Último pago'</t>
+          <t>Consulta con montos ('$') y perfil con 'Último pago'</t>
         </is>
       </c>
       <c r="F229" s="3" t="inlineStr">
         <is>
-          <t>'Último pago' visible: True</t>
+          <t>Montos en la consulta: True; 'Último pago' en el perfil: True</t>
         </is>
       </c>
       <c r="G229" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: PreNominaIntegracionViewTest.test_perfil_muestra_ultimo_pago</t>
+          <t>Prueba automatizada: IntegracionNominaTest.test_ciclo_completo_empleado_ve_pago</t>
         </is>
       </c>
       <c r="H229" s="3" t="inlineStr">
@@ -10105,32 +10105,32 @@
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>RF-013</t>
+          <t>RF-012</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>Integración: permisos de la bandeja de aprobación por rol.</t>
+          <t>Validar que el perfil del empleado muestre su último pago.</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>GET /nomina/bandeja/ con cada rol y sin sesión</t>
+          <t>Pre-nómina aprobada; el empleado abre su perfil</t>
         </is>
       </c>
       <c r="E230" s="2" t="inlineStr">
         <is>
-          <t>Gerente 403; Auxiliar 200; Vendedor 403; anónimo 302</t>
+          <t>El perfil muestra 'Último pago'</t>
         </is>
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>Gerente 403; Auxiliar 200; Vendedor 403; anónimo 302</t>
+          <t>'Último pago' visible: True</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: IntegracionNominaTest.test_permisos_bandeja</t>
+          <t>Prueba automatizada: PreNominaIntegracionViewTest.test_perfil_muestra_ultimo_pago</t>
         </is>
       </c>
       <c r="H230" s="2" t="inlineStr">
@@ -10152,27 +10152,27 @@
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Integración: permisos del cálculo de nómina por rol.</t>
+          <t>Integración: permisos de la bandeja de aprobación por rol.</t>
         </is>
       </c>
       <c r="D231" s="3" t="inlineStr">
         <is>
-          <t>GET /nomina/calculo/ con cada rol y sin sesión</t>
+          <t>GET /nomina/bandeja/ con cada rol y sin sesión</t>
         </is>
       </c>
       <c r="E231" s="3" t="inlineStr">
         <is>
-          <t>Gerente 200; Auxiliar 403; Vendedor 403; anónimo 302</t>
+          <t>Gerente 403; Auxiliar 200; Vendedor 403; anónimo 302</t>
         </is>
       </c>
       <c r="F231" s="3" t="inlineStr">
         <is>
-          <t>Gerente 200; Auxiliar 403; Vendedor 403; anónimo 302</t>
+          <t>Gerente 403; Auxiliar 200; Vendedor 403; anónimo 302</t>
         </is>
       </c>
       <c r="G231" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: IntegracionNominaTest.test_permisos_calculo</t>
+          <t>Prueba automatizada: IntegracionNominaTest.test_permisos_bandeja</t>
         </is>
       </c>
       <c r="H231" s="3" t="inlineStr">
@@ -10194,27 +10194,27 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>Integración: permisos del detalle de pre-nómina por rol.</t>
+          <t>Integración: permisos del cálculo de nómina por rol.</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>GET detalle de pre-nómina con cada rol y sin sesión</t>
+          <t>GET /nomina/calculo/ con cada rol y sin sesión</t>
         </is>
       </c>
       <c r="E232" s="2" t="inlineStr">
         <is>
-          <t>Gerente 403; Auxiliar 200; Vendedor 403; anónimo 302</t>
+          <t>Gerente 200; Auxiliar 403; Vendedor 403; anónimo 302</t>
         </is>
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>Gerente 403; Auxiliar 200; Vendedor 403; anónimo 302</t>
+          <t>Gerente 200; Auxiliar 403; Vendedor 403; anónimo 302</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: IntegracionNominaTest.test_permisos_detalle_prenomina</t>
+          <t>Prueba automatizada: IntegracionNominaTest.test_permisos_calculo</t>
         </is>
       </c>
       <c r="H232" s="2" t="inlineStr">
@@ -10236,27 +10236,27 @@
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Integración: permisos de la ventana Novedades por rol.</t>
+          <t>Integración: permisos del detalle de pre-nómina por rol.</t>
         </is>
       </c>
       <c r="D233" s="3" t="inlineStr">
         <is>
-          <t>GET /nomina/novedades/ con cada rol y sin sesión</t>
+          <t>GET detalle de pre-nómina con cada rol y sin sesión</t>
         </is>
       </c>
       <c r="E233" s="3" t="inlineStr">
         <is>
-          <t>Gerente 200; Auxiliar 403; Vendedor 403; anónimo 302</t>
+          <t>Gerente 403; Auxiliar 200; Vendedor 403; anónimo 302</t>
         </is>
       </c>
       <c r="F233" s="3" t="inlineStr">
         <is>
-          <t>Gerente 200; Auxiliar 403; Vendedor 403; anónimo 302</t>
+          <t>Gerente 403; Auxiliar 200; Vendedor 403; anónimo 302</t>
         </is>
       </c>
       <c r="G233" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: IntegracionNominaTest.test_permisos_novedades</t>
+          <t>Prueba automatizada: IntegracionNominaTest.test_permisos_detalle_prenomina</t>
         </is>
       </c>
       <c r="H233" s="3" t="inlineStr">
@@ -10278,27 +10278,27 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>Integración: permisos de la pantalla de reportes por rol.</t>
+          <t>Integración: permisos de la ventana Novedades por rol.</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>GET /nomina/reportes/ con cada rol y sin sesión</t>
+          <t>GET /nomina/novedades/ con cada rol y sin sesión</t>
         </is>
       </c>
       <c r="E234" s="2" t="inlineStr">
         <is>
-          <t>Gerente 200; Auxiliar 200; Vendedor 403; anónimo 302</t>
+          <t>Gerente 200; Auxiliar 403; Vendedor 403; anónimo 302</t>
         </is>
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>Gerente 200; Auxiliar 200; Vendedor 403; anónimo 302</t>
+          <t>Gerente 200; Auxiliar 403; Vendedor 403; anónimo 302</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: IntegracionNominaTest.test_permisos_reporte_mensual</t>
+          <t>Prueba automatizada: IntegracionNominaTest.test_permisos_novedades</t>
         </is>
       </c>
       <c r="H234" s="2" t="inlineStr">
@@ -10320,12 +10320,12 @@
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Integración: permisos de la descarga del PDF por rol.</t>
+          <t>Integración: permisos de la pantalla de reportes por rol.</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
         <is>
-          <t>GET /nomina/reportes/pdf/ con cada rol y sin sesión</t>
+          <t>GET /nomina/reportes/ con cada rol y sin sesión</t>
         </is>
       </c>
       <c r="E235" s="3" t="inlineStr">
@@ -10340,7 +10340,7 @@
       </c>
       <c r="G235" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: IntegracionNominaTest.test_permisos_reporte_pdf</t>
+          <t>Prueba automatizada: IntegracionNominaTest.test_permisos_reporte_mensual</t>
         </is>
       </c>
       <c r="H235" s="3" t="inlineStr">
@@ -10357,32 +10357,32 @@
       </c>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>RF-014</t>
+          <t>RF-013</t>
         </is>
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>Validar la creación de un rol nuevo.</t>
+          <t>Integración: permisos de la descarga del PDF por rol.</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>nombre del rol: 'Supervisor'</t>
+          <t>GET /nomina/reportes/pdf/ con cada rol y sin sesión</t>
         </is>
       </c>
       <c r="E236" s="2" t="inlineStr">
         <is>
-          <t>El rol Supervisor existe</t>
+          <t>Gerente 200; Auxiliar 200; Vendedor 403; anónimo 302</t>
         </is>
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>Rol creado: True</t>
+          <t>Gerente 200; Auxiliar 200; Vendedor 403; anónimo 302</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: GestionRolesT61Test.test_crear_rol</t>
+          <t>Prueba automatizada: IntegracionNominaTest.test_permisos_reporte_pdf</t>
         </is>
       </c>
       <c r="H236" s="2" t="inlineStr">
@@ -10404,27 +10404,27 @@
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Validar que no se cree un rol con nombre repetido.</t>
+          <t>Validar la creación de un rol nuevo.</t>
         </is>
       </c>
       <c r="D237" s="3" t="inlineStr">
         <is>
-          <t>nombre del rol: 'Vendedor'</t>
+          <t>nombre del rol: 'Supervisor'</t>
         </is>
       </c>
       <c r="E237" s="3" t="inlineStr">
         <is>
-          <t>Ya existe un rol con ese nombre.</t>
+          <t>El rol Supervisor existe</t>
         </is>
       </c>
       <c r="F237" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200; mensaje visible: True</t>
+          <t>Rol creado: True</t>
         </is>
       </c>
       <c r="G237" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: GestionRolesT61Test.test_crear_rol_duplicado_muestra_mensaje</t>
+          <t>Prueba automatizada: GestionRolesT61Test.test_crear_rol</t>
         </is>
       </c>
       <c r="H237" s="3" t="inlineStr">
@@ -10446,27 +10446,27 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>Validar la eliminación de un rol sin usuarios.</t>
+          <t>Validar que no se cree un rol con nombre repetido.</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>rol 'Temporal' sin usuarios</t>
+          <t>nombre del rol: 'Vendedor'</t>
         </is>
       </c>
       <c r="E238" s="2" t="inlineStr">
         <is>
-          <t>El rol deja de existir</t>
+          <t>Ya existe un rol con ese nombre.</t>
         </is>
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>Rol sigue existiendo: False</t>
+          <t>HTTP 200; mensaje visible: True</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: GestionRolesT61Test.test_eliminar_rol_vacio</t>
+          <t>Prueba automatizada: GestionRolesT61Test.test_crear_rol_duplicado_muestra_mensaje</t>
         </is>
       </c>
       <c r="H238" s="2" t="inlineStr">
@@ -10488,27 +10488,27 @@
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Validar que no se pueda eliminar un rol base del sistema.</t>
+          <t>Validar la eliminación de un rol sin usuarios.</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
         <is>
-          <t>eliminar rol 'Vendedor'</t>
+          <t>rol 'Temporal' sin usuarios</t>
         </is>
       </c>
       <c r="E239" s="3" t="inlineStr">
         <is>
-          <t>No se puede eliminar el rol Vendedor porque es un rol base del sistema.</t>
+          <t>El rol deja de existir</t>
         </is>
       </c>
       <c r="F239" s="3" t="inlineStr">
         <is>
-          <t>Mensaje visible: True; rol conservado: True</t>
+          <t>Rol sigue existiendo: False</t>
         </is>
       </c>
       <c r="G239" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: GestionRolesT61Test.test_no_elimina_rol_base</t>
+          <t>Prueba automatizada: GestionRolesT61Test.test_eliminar_rol_vacio</t>
         </is>
       </c>
       <c r="H239" s="3" t="inlineStr">
@@ -10530,17 +10530,17 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>Validar que no se pueda eliminar un rol con usuarios asignados.</t>
+          <t>Validar que no se pueda eliminar un rol base del sistema.</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>rol 'Con usuarios' con 1 usuario</t>
+          <t>eliminar rol 'Vendedor'</t>
         </is>
       </c>
       <c r="E240" s="2" t="inlineStr">
         <is>
-          <t>No se puede eliminar el rol Con usuarios porque tiene 1 usuario(s) asignado(s).</t>
+          <t>No se puede eliminar el rol Vendedor porque es un rol base del sistema.</t>
         </is>
       </c>
       <c r="F240" s="2" t="inlineStr">
@@ -10550,7 +10550,7 @@
       </c>
       <c r="G240" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: GestionRolesT61Test.test_no_elimina_rol_con_usuarios_asignados</t>
+          <t>Prueba automatizada: GestionRolesT61Test.test_no_elimina_rol_base</t>
         </is>
       </c>
       <c r="H240" s="2" t="inlineStr">
@@ -10572,27 +10572,27 @@
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Validar que nombre de rol rechace números.</t>
+          <t>Validar que no se pueda eliminar un rol con usuarios asignados.</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
         <is>
-          <t>rol: 'Rol2'</t>
+          <t>rol 'Con usuarios' con 1 usuario</t>
         </is>
       </c>
       <c r="E241" s="3" t="inlineStr">
         <is>
-          <t>El formulario informa que el nombre solo admite letras y espacios.</t>
+          <t>No se puede eliminar el rol Con usuarios porque tiene 1 usuario(s) asignado(s).</t>
         </is>
       </c>
       <c r="F241" s="3" t="inlineStr">
         <is>
-          <t>Mensaje mostrado: El nombre del rol solo puede contener letras y espacios.</t>
+          <t>Mensaje visible: True; rol conservado: True</t>
         </is>
       </c>
       <c r="G241" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ValidacionesGestionUsuarioTest.test_rol_nombre_con_numero</t>
+          <t>Prueba automatizada: GestionRolesT61Test.test_no_elimina_rol_con_usuarios_asignados</t>
         </is>
       </c>
       <c r="H241" s="3" t="inlineStr">
@@ -10614,27 +10614,27 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>Validar que nombre de rol duplicado sea rechazado.</t>
+          <t>Validar que nombre de rol rechace números.</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>rol: 'gerente'; ya existe 'Gerente'</t>
+          <t>rol: 'Rol2'</t>
         </is>
       </c>
       <c r="E242" s="2" t="inlineStr">
         <is>
-          <t>El formulario informa que el rol ya existe.</t>
+          <t>El formulario informa que el nombre solo admite letras y espacios.</t>
         </is>
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>Mensaje mostrado: Ya existe un rol con ese nombre.</t>
+          <t>Mensaje mostrado: El nombre del rol solo puede contener letras y espacios.</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ValidacionesGestionUsuarioTest.test_rol_nombre_duplicado</t>
+          <t>Prueba automatizada: ValidacionesGestionUsuarioTest.test_rol_nombre_con_numero</t>
         </is>
       </c>
       <c r="H242" s="2" t="inlineStr">
@@ -10656,27 +10656,27 @@
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Validar edición de rol por gerente.</t>
+          <t>Validar que nombre de rol duplicado sea rechazado.</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
         <is>
-          <t>POST editar rol Vendedor sin permisos</t>
+          <t>rol: 'gerente'; ya existe 'Gerente'</t>
         </is>
       </c>
       <c r="E243" s="3" t="inlineStr">
         <is>
-          <t>La respuesta HTTP 302.</t>
+          <t>El formulario informa que el rol ya existe.</t>
         </is>
       </c>
       <c r="F243" s="3" t="inlineStr">
         <is>
-          <t>HTTP 302; redirige a /roles/</t>
+          <t>Mensaje mostrado: Ya existe un rol con ese nombre.</t>
         </is>
       </c>
       <c r="G243" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: GestionUsuariosTest.test_gerente_edita_rol</t>
+          <t>Prueba automatizada: ValidacionesGestionUsuarioTest.test_rol_nombre_duplicado</t>
         </is>
       </c>
       <c r="H243" s="3" t="inlineStr">
@@ -10693,32 +10693,32 @@
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>RF-015</t>
+          <t>RF-014</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>Validar que un usuario pueda registrarse con dos roles.</t>
+          <t>Validar edición de rol por gerente.</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>Registro con roles Vendedor y Auxiliar Administrativo</t>
+          <t>POST editar rol Vendedor sin permisos</t>
         </is>
       </c>
       <c r="E244" s="2" t="inlineStr">
         <is>
-          <t>Roles: 'Auxiliar Administrativo, Vendedor'</t>
+          <t>La respuesta HTTP 302.</t>
         </is>
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>Roles asignados: Auxiliar Administrativo, Vendedor</t>
+          <t>HTTP 302; redirige a /roles/</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: RolesMultiplesT61Test.test_crear_usuario_con_dos_roles</t>
+          <t>Prueba automatizada: GestionUsuariosTest.test_gerente_edita_rol</t>
         </is>
       </c>
       <c r="H244" s="2" t="inlineStr">
@@ -10740,27 +10740,27 @@
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Validar que no se registre un usuario sin roles.</t>
+          <t>Validar que un usuario pueda registrarse con dos roles.</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
         <is>
-          <t>Registro sin seleccionar roles</t>
+          <t>Registro con roles Vendedor y Auxiliar Administrativo</t>
         </is>
       </c>
       <c r="E245" s="3" t="inlineStr">
         <is>
-          <t>Selecciona al menos un rol para el usuario.</t>
+          <t>Roles: 'Auxiliar Administrativo, Vendedor'</t>
         </is>
       </c>
       <c r="F245" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200; mensaje visible: True</t>
+          <t>Roles asignados: Auxiliar Administrativo, Vendedor</t>
         </is>
       </c>
       <c r="G245" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: RolesMultiplesT61Test.test_crear_usuario_sin_roles_muestra_mensaje</t>
+          <t>Prueba automatizada: RolesMultiplesT61Test.test_crear_usuario_con_dos_roles</t>
         </is>
       </c>
       <c r="H245" s="3" t="inlineStr">
@@ -10782,27 +10782,27 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>Validar que un usuario con dos roles acceda a la bandeja del Auxiliar.</t>
+          <t>Validar que no se registre un usuario sin roles.</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
         <is>
-          <t>Usuario Vendedor + Auxiliar abre la bandeja de aprobación</t>
+          <t>Registro sin seleccionar roles</t>
         </is>
       </c>
       <c r="E246" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Selecciona al menos un rol para el usuario.</t>
         </is>
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>HTTP 200; mensaje visible: True</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: RolesMultiplesT61Test.test_dos_roles_accede_bandeja</t>
+          <t>Prueba automatizada: RolesMultiplesT61Test.test_crear_usuario_sin_roles_muestra_mensaje</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
@@ -10824,12 +10824,12 @@
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Validar que un usuario con dos roles acceda a la consulta de nómina del Vendedor.</t>
+          <t>Validar que un usuario con dos roles acceda a la bandeja del Auxiliar.</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
         <is>
-          <t>Usuario Vendedor + Auxiliar abre la consulta de nómina</t>
+          <t>Usuario Vendedor + Auxiliar abre la bandeja de aprobación</t>
         </is>
       </c>
       <c r="E247" s="3" t="inlineStr">
@@ -10844,7 +10844,7 @@
       </c>
       <c r="G247" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: RolesMultiplesT61Test.test_dos_roles_accede_consulta</t>
+          <t>Prueba automatizada: RolesMultiplesT61Test.test_dos_roles_accede_bandeja</t>
         </is>
       </c>
       <c r="H247" s="3" t="inlineStr">
@@ -10866,27 +10866,27 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>Validar que un usuario pueda tener varios roles.</t>
+          <t>Validar que un usuario con dos roles acceda a la consulta de nómina del Vendedor.</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>roles: Vendedor y Auxiliar</t>
+          <t>Usuario Vendedor + Auxiliar abre la consulta de nómina</t>
         </is>
       </c>
       <c r="E248" s="2" t="inlineStr">
         <is>
-          <t>El formulario acepta ambos roles.</t>
+          <t>HTTP 200</t>
         </is>
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>Formulario válido: True</t>
+          <t>HTTP 200</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ValidacionesGestionUsuarioTest.test_varios_roles_permitidos</t>
+          <t>Prueba automatizada: RolesMultiplesT61Test.test_dos_roles_accede_consulta</t>
         </is>
       </c>
       <c r="H248" s="2" t="inlineStr">
@@ -10903,32 +10903,32 @@
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>RF-016</t>
+          <t>RF-015</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Validar el filtro de usuarios por estado.</t>
+          <t>Validar que un usuario pueda tener varios roles.</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
         <is>
-          <t>estado: INACTIVO</t>
+          <t>roles: Vendedor y Auxiliar</t>
         </is>
       </c>
       <c r="E249" s="3" t="inlineStr">
         <is>
-          <t>AmbosFiltro y AuxFiltro</t>
+          <t>El formulario acepta ambos roles.</t>
         </is>
       </c>
       <c r="F249" s="3" t="inlineStr">
         <is>
-          <t>Usuarios listados: ['AmbosFiltro', 'AuxFiltro']</t>
+          <t>Formulario válido: True</t>
         </is>
       </c>
       <c r="G249" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: FiltrosUsuariosT61Test.test_filtro_por_estado</t>
+          <t>Prueba automatizada: ValidacionesGestionUsuarioTest.test_varios_roles_permitidos</t>
         </is>
       </c>
       <c r="H249" s="3" t="inlineStr">
@@ -10950,27 +10950,27 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>Validar el filtro por nombre parcial sin distinguir mayúsculas.</t>
+          <t>Validar el filtro de usuarios por estado.</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
         <is>
-          <t>nombre: 'aNa mA'</t>
+          <t>estado: INACTIVO</t>
         </is>
       </c>
       <c r="E250" s="2" t="inlineStr">
         <is>
-          <t>AnaFiltro</t>
+          <t>AmbosFiltro y AuxFiltro</t>
         </is>
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>Usuarios listados: ['AnaFiltro']</t>
+          <t>Usuarios listados: ['AmbosFiltro', 'AuxFiltro']</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: FiltrosUsuariosT61Test.test_filtro_por_nombre_parcial_sin_distinguir_mayusculas</t>
+          <t>Prueba automatizada: FiltrosUsuariosT61Test.test_filtro_por_estado</t>
         </is>
       </c>
       <c r="H250" s="2" t="inlineStr">
@@ -10992,27 +10992,27 @@
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Validar el filtro de usuarios por rol.</t>
+          <t>Validar el filtro por nombre parcial sin distinguir mayúsculas.</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
         <is>
-          <t>rol: Vendedor</t>
+          <t>nombre: 'aNa mA'</t>
         </is>
       </c>
       <c r="E251" s="3" t="inlineStr">
         <is>
-          <t>AmbosFiltro y AnaFiltro</t>
+          <t>AnaFiltro</t>
         </is>
       </c>
       <c r="F251" s="3" t="inlineStr">
         <is>
-          <t>Usuarios listados: ['AmbosFiltro', 'AnaFiltro']</t>
+          <t>Usuarios listados: ['AnaFiltro']</t>
         </is>
       </c>
       <c r="G251" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: FiltrosUsuariosT61Test.test_filtro_por_rol</t>
+          <t>Prueba automatizada: FiltrosUsuariosT61Test.test_filtro_por_nombre_parcial_sin_distinguir_mayusculas</t>
         </is>
       </c>
       <c r="H251" s="3" t="inlineStr">
@@ -11034,27 +11034,27 @@
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>Validar la combinación de filtros de rol, estado y nombre.</t>
+          <t>Validar el filtro de usuarios por rol.</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
         <is>
-          <t>rol: Auxiliar; estado: INACTIVO; nombre: 'ana'</t>
+          <t>rol: Vendedor</t>
         </is>
       </c>
       <c r="E252" s="2" t="inlineStr">
         <is>
-          <t>AmbosFiltro</t>
+          <t>AmbosFiltro y AnaFiltro</t>
         </is>
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>Usuarios listados: ['AmbosFiltro']</t>
+          <t>Usuarios listados: ['AmbosFiltro', 'AnaFiltro']</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: FiltrosUsuariosT61Test.test_filtros_combinados</t>
+          <t>Prueba automatizada: FiltrosUsuariosT61Test.test_filtro_por_rol</t>
         </is>
       </c>
       <c r="H252" s="2" t="inlineStr">
@@ -11076,27 +11076,27 @@
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>Validar que el filtro de nombre rechace caracteres especiales.</t>
+          <t>Validar la combinación de filtros de rol, estado y nombre.</t>
         </is>
       </c>
       <c r="D253" s="3" t="inlineStr">
         <is>
-          <t>nombre: '&lt;'</t>
+          <t>rol: Auxiliar; estado: INACTIVO; nombre: 'ana'</t>
         </is>
       </c>
       <c r="E253" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200 con: El filtro de nombre contiene caracteres no permitidos.</t>
+          <t>AmbosFiltro</t>
         </is>
       </c>
       <c r="F253" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200; mensaje visible: True</t>
+          <t>Usuarios listados: ['AmbosFiltro']</t>
         </is>
       </c>
       <c r="G253" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: FiltrosUsuariosT61Test.test_nombre_con_menor_muestra_error_y_responde_200</t>
+          <t>Prueba automatizada: FiltrosUsuariosT61Test.test_filtros_combinados</t>
         </is>
       </c>
       <c r="H253" s="3" t="inlineStr">
@@ -11113,32 +11113,32 @@
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>RF-017</t>
+          <t>RF-016</t>
         </is>
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>Validar que el cambio de contraseña quede en la auditoría.</t>
+          <t>Validar que el filtro de nombre rechace caracteres especiales.</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>Cambio de contraseña válido</t>
+          <t>nombre: '&lt;'</t>
         </is>
       </c>
       <c r="E254" s="2" t="inlineStr">
         <is>
-          <t>Registro 'Cambió su contraseña' del usuario</t>
+          <t>HTTP 200 con: El filtro de nombre contiene caracteres no permitidos.</t>
         </is>
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>Auditoría registrada: True</t>
+          <t>HTTP 200; mensaje visible: True</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: CambioContrasenaT61Test.test_cambio_valido_registra_auditoria</t>
+          <t>Prueba automatizada: FiltrosUsuariosT61Test.test_nombre_con_menor_muestra_error_y_responde_200</t>
         </is>
       </c>
       <c r="H254" s="2" t="inlineStr">
@@ -11160,17 +11160,17 @@
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>Validar que la creación de un rol quede en la auditoría.</t>
+          <t>Validar que el cambio de contraseña quede en la auditoría.</t>
         </is>
       </c>
       <c r="D255" s="3" t="inlineStr">
         <is>
-          <t>nombre del rol: 'Supervisor'</t>
+          <t>Cambio de contraseña válido</t>
         </is>
       </c>
       <c r="E255" s="3" t="inlineStr">
         <is>
-          <t>Registro CREAR 'Creó el rol Supervisor'</t>
+          <t>Registro 'Cambió su contraseña' del usuario</t>
         </is>
       </c>
       <c r="F255" s="3" t="inlineStr">
@@ -11180,7 +11180,7 @@
       </c>
       <c r="G255" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: GestionRolesT61Test.test_crear_rol_registra_auditoria</t>
+          <t>Prueba automatizada: CambioContrasenaT61Test.test_cambio_valido_registra_auditoria</t>
         </is>
       </c>
       <c r="H255" s="3" t="inlineStr">
@@ -11202,17 +11202,17 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>Validar que la eliminación de un rol quede en la auditoría.</t>
+          <t>Validar que la creación de un rol quede en la auditoría.</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>rol 'Temporal' eliminado</t>
+          <t>nombre del rol: 'Supervisor'</t>
         </is>
       </c>
       <c r="E256" s="2" t="inlineStr">
         <is>
-          <t>Registro ELIMINAR 'Eliminó el rol Temporal'</t>
+          <t>Registro CREAR 'Creó el rol Supervisor'</t>
         </is>
       </c>
       <c r="F256" s="2" t="inlineStr">
@@ -11222,7 +11222,7 @@
       </c>
       <c r="G256" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: GestionRolesT61Test.test_eliminar_rol_vacio_registra_auditoria</t>
+          <t>Prueba automatizada: GestionRolesT61Test.test_crear_rol_registra_auditoria</t>
         </is>
       </c>
       <c r="H256" s="2" t="inlineStr">
@@ -11244,27 +11244,27 @@
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>Validar que un intento de acceso fallido quede en la auditoría.</t>
+          <t>Validar que la eliminación de un rol quede en la auditoría.</t>
         </is>
       </c>
       <c r="D257" s="3" t="inlineStr">
         <is>
-          <t>correo válido; contraseña 'Incorrecta1'</t>
+          <t>rol 'Temporal' eliminado</t>
         </is>
       </c>
       <c r="E257" s="3" t="inlineStr">
         <is>
-          <t>Registro ERROR_ACCESO con el correo usado</t>
+          <t>Registro ELIMINAR 'Eliminó el rol Temporal'</t>
         </is>
       </c>
       <c r="F257" s="3" t="inlineStr">
         <is>
-          <t>Auditoría ERROR_ACCESO registrada: True</t>
+          <t>Auditoría registrada: True</t>
         </is>
       </c>
       <c r="G257" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: LoginT61Test.test_contrasena_incorrecta_crea_auditoria</t>
+          <t>Prueba automatizada: GestionRolesT61Test.test_eliminar_rol_vacio_registra_auditoria</t>
         </is>
       </c>
       <c r="H257" s="3" t="inlineStr">
@@ -11286,27 +11286,27 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>Validar mensaje de fecha inválida en auditoría.</t>
+          <t>Validar que un intento de acceso fallido quede en la auditoría.</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t>GET /auditoria/?fecha=xx como Gerente</t>
+          <t>correo válido; contraseña 'Incorrecta1'</t>
         </is>
       </c>
       <c r="E258" s="2" t="inlineStr">
         <is>
-          <t>La respuesta muestra Escribe una fecha válida en el filtro.</t>
+          <t>Registro ERROR_ACCESO con el correo usado</t>
         </is>
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>Mensaje mostrado: Escribe una fecha válida en el filtro.</t>
+          <t>Auditoría ERROR_ACCESO registrada: True</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: AuditoriaFiltroValidacionTest.test_fecha_invalida_muestra_mensaje</t>
+          <t>Prueba automatizada: LoginT61Test.test_contrasena_incorrecta_crea_auditoria</t>
         </is>
       </c>
       <c r="H258" s="2" t="inlineStr">
@@ -11328,7 +11328,7 @@
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>Validar respuesta HTTP del filtro de auditoría con fecha inválida.</t>
+          <t>Validar mensaje de fecha inválida en auditoría.</t>
         </is>
       </c>
       <c r="D259" s="3" t="inlineStr">
@@ -11338,17 +11338,17 @@
       </c>
       <c r="E259" s="3" t="inlineStr">
         <is>
-          <t>La respuesta es HTTP 200.</t>
+          <t>La respuesta muestra Escribe una fecha válida en el filtro.</t>
         </is>
       </c>
       <c r="F259" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Mensaje mostrado: Escribe una fecha válida en el filtro.</t>
         </is>
       </c>
       <c r="G259" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: AuditoriaFiltroValidacionTest.test_fecha_invalida_responde_200</t>
+          <t>Prueba automatizada: AuditoriaFiltroValidacionTest.test_fecha_invalida_muestra_mensaje</t>
         </is>
       </c>
       <c r="H259" s="3" t="inlineStr">
@@ -11370,27 +11370,27 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>Validar representación textual de auditoría.</t>
+          <t>Validar respuesta HTTP del filtro de auditoría con fecha inválida.</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>registro con detalle 'Prueba de formato'</t>
+          <t>GET /auditoria/?fecha=xx como Gerente</t>
         </is>
       </c>
       <c r="E260" s="2" t="inlineStr">
         <is>
-          <t>La representación incluye Prueba de formato.</t>
+          <t>La respuesta es HTTP 200.</t>
         </is>
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>Representación: gerente-t16 (ID: 85 - Identificacion: None - Estado: ACTIVO) - Crear (Prueba de formato)</t>
+          <t>HTTP 200</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: GestionUsuariosTest.test_auditoria_se_formatea</t>
+          <t>Prueba automatizada: AuditoriaFiltroValidacionTest.test_fecha_invalida_responde_200</t>
         </is>
       </c>
       <c r="H260" s="2" t="inlineStr">
@@ -11412,27 +11412,27 @@
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>Validar auditoría al crear usuario.</t>
+          <t>Validar representación textual de auditoría.</t>
         </is>
       </c>
       <c r="D261" s="3" t="inlineStr">
         <is>
-          <t>POST de creación de vendedor-t16 por gerente</t>
+          <t>registro con detalle 'Prueba de formato'</t>
         </is>
       </c>
       <c r="E261" s="3" t="inlineStr">
         <is>
-          <t>Auditoría registra acción CREAR y el nombre Violeta Prueba.</t>
+          <t>La representación incluye Prueba de formato.</t>
         </is>
       </c>
       <c r="F261" s="3" t="inlineStr">
         <is>
-          <t>Registro de auditoría encontrado: True</t>
+          <t>Representación: gerente-t16 (ID: 87 - Identificacion: None - Estado: ACTIVO) - Crear (Prueba de formato)</t>
         </is>
       </c>
       <c r="G261" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: GestionUsuariosTest.test_crear_usuario_registra_auditoria</t>
+          <t>Prueba automatizada: GestionUsuariosTest.test_auditoria_se_formatea</t>
         </is>
       </c>
       <c r="H261" s="3" t="inlineStr">
@@ -11454,17 +11454,17 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>Validar auditoría al eliminar usuario.</t>
+          <t>Validar auditoría al crear usuario.</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
         <is>
-          <t>POST eliminar usuario vendedor-t16 por gerente</t>
+          <t>POST de creación de vendedor-t16 por gerente</t>
         </is>
       </c>
       <c r="E262" s="2" t="inlineStr">
         <is>
-          <t>Auditoría registra acción ELIMINAR y el username vendedor-t16.</t>
+          <t>Auditoría registra acción CREAR y el nombre Violeta Prueba.</t>
         </is>
       </c>
       <c r="F262" s="2" t="inlineStr">
@@ -11474,7 +11474,7 @@
       </c>
       <c r="G262" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: GestionUsuariosTest.test_eliminar_usuario_registra_auditoria</t>
+          <t>Prueba automatizada: GestionUsuariosTest.test_crear_usuario_registra_auditoria</t>
         </is>
       </c>
       <c r="H262" s="2" t="inlineStr">
@@ -11496,27 +11496,27 @@
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>Integración: el ciclo completo deja rastro en la auditoría.</t>
+          <t>Validar auditoría al eliminar usuario.</t>
         </is>
       </c>
       <c r="D263" s="3" t="inlineStr">
         <is>
-          <t>Ciclo completo y exportación del PDF</t>
+          <t>POST eliminar usuario vendedor-t16 por gerente</t>
         </is>
       </c>
       <c r="E263" s="3" t="inlineStr">
         <is>
-          <t>Auditoría con CREAR usuario, ACTUALIZAR bonificación, ACTUALIZAR aceptación, CALCULAR y EXPORTAR</t>
+          <t>Auditoría registra acción ELIMINAR y el username vendedor-t16.</t>
         </is>
       </c>
       <c r="F263" s="3" t="inlineStr">
         <is>
-          <t>Acciones registradas: 5 de 5; faltantes: ninguna</t>
+          <t>Registro de auditoría encontrado: True</t>
         </is>
       </c>
       <c r="G263" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: IntegracionNominaTest.test_ciclo_completo_auditoria</t>
+          <t>Prueba automatizada: GestionUsuariosTest.test_eliminar_usuario_registra_auditoria</t>
         </is>
       </c>
       <c r="H263" s="3" t="inlineStr">
@@ -11538,27 +11538,27 @@
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>Validar que la exportación del PDF quede en la auditoría.</t>
+          <t>Integración: el ciclo completo deja rastro en la auditoría.</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>Gerente descarga el PDF de 2026-09</t>
+          <t>Ciclo completo y exportación del PDF</t>
         </is>
       </c>
       <c r="E264" s="2" t="inlineStr">
         <is>
-          <t>Registro de auditoría con acción EXPORTAR del Gerente</t>
+          <t>Auditoría con CREAR usuario, ACTUALIZAR bonificación, ACTUALIZAR aceptación, CALCULAR y EXPORTAR</t>
         </is>
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>Auditoría EXPORTAR registrada: True</t>
+          <t>Acciones registradas: 5 de 5; faltantes: ninguna</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ReportePDFViewTest.test_exportar_pdf_registra_auditoria</t>
+          <t>Prueba automatizada: IntegracionNominaTest.test_ciclo_completo_auditoria</t>
         </is>
       </c>
       <c r="H264" s="2" t="inlineStr">
@@ -11575,32 +11575,32 @@
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>RNF-001</t>
+          <t>RF-017</t>
         </is>
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>Validar que las contraseñas almacenadas usen algoritmos de hash.</t>
+          <t>Validar que la exportación del PDF quede en la auditoría.</t>
         </is>
       </c>
       <c r="D265" s="3" t="inlineStr">
         <is>
-          <t>Usuario creado mediante create_user</t>
+          <t>Gerente descarga el PDF de 2026-09</t>
         </is>
       </c>
       <c r="E265" s="3" t="inlineStr">
         <is>
-          <t>Todas las contraseñas empiezan con prefijo de hash</t>
+          <t>Registro de auditoría con acción EXPORTAR del Gerente</t>
         </is>
       </c>
       <c r="F265" s="3" t="inlineStr">
         <is>
-          <t>Se encontraron 1 usuarios y todos usan contraseñas con hash.</t>
+          <t>Auditoría EXPORTAR registrada: True</t>
         </is>
       </c>
       <c r="G265" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: RendimientoNominaTest.test_contrasenas_de_usuarios_no_estan_en_texto_plano</t>
+          <t>Prueba automatizada: ReportePDFViewTest.test_exportar_pdf_registra_auditoria</t>
         </is>
       </c>
       <c r="H265" s="3" t="inlineStr">
@@ -11617,32 +11617,32 @@
       </c>
       <c r="B266" s="2" t="inlineStr">
         <is>
-          <t>RNF-003</t>
+          <t>RNF-001</t>
         </is>
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>Validar que un Vendedor no pueda crear roles.</t>
+          <t>Validar que las contraseñas almacenadas usen algoritmos de hash.</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
         <is>
-          <t>Vendedor envía rol 'Supervisor'</t>
+          <t>Usuario creado mediante create_user</t>
         </is>
       </c>
       <c r="E266" s="2" t="inlineStr">
         <is>
-          <t>HTTP 403</t>
+          <t>Todas las contraseñas empiezan con prefijo de hash</t>
         </is>
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>HTTP 403</t>
+          <t>Se encontraron 1 usuarios y todos usan contraseñas con hash.</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: GestionRolesT61Test.test_vendedor_no_puede_crear_roles</t>
+          <t>Prueba automatizada: RendimientoNominaTest.test_contrasenas_de_usuarios_no_estan_en_texto_plano</t>
         </is>
       </c>
       <c r="H266" s="2" t="inlineStr">
@@ -11664,12 +11664,12 @@
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>Validar que un Vendedor no pueda eliminar roles.</t>
+          <t>Validar que un Vendedor no pueda crear roles.</t>
         </is>
       </c>
       <c r="D267" s="3" t="inlineStr">
         <is>
-          <t>Vendedor intenta eliminar el rol Gerente</t>
+          <t>Vendedor envía rol 'Supervisor'</t>
         </is>
       </c>
       <c r="E267" s="3" t="inlineStr">
@@ -11684,7 +11684,7 @@
       </c>
       <c r="G267" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: GestionRolesT61Test.test_vendedor_no_puede_eliminar_roles</t>
+          <t>Prueba automatizada: GestionRolesT61Test.test_vendedor_no_puede_crear_roles</t>
         </is>
       </c>
       <c r="H267" s="3" t="inlineStr">
@@ -11706,12 +11706,12 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>Validar que un Vendedor no acceda a la ventana Novedades.</t>
+          <t>Validar que un Vendedor no pueda eliminar roles.</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>Vendedor abre /nomina/novedades/</t>
+          <t>Vendedor intenta eliminar el rol Gerente</t>
         </is>
       </c>
       <c r="E268" s="2" t="inlineStr">
@@ -11726,7 +11726,7 @@
       </c>
       <c r="G268" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: NovedadesViewTest.test_novedades_restringe_vendedor</t>
+          <t>Prueba automatizada: GestionRolesT61Test.test_vendedor_no_puede_eliminar_roles</t>
         </is>
       </c>
       <c r="H268" s="2" t="inlineStr">
@@ -11748,27 +11748,27 @@
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>Validar que solo el Auxiliar pueda abrir el detalle de la pre-nómina.</t>
+          <t>Validar que un Vendedor no acceda a la ventana Novedades.</t>
         </is>
       </c>
       <c r="D269" s="3" t="inlineStr">
         <is>
-          <t>Gerente y Vendedor abren el detalle</t>
+          <t>Vendedor abre /nomina/novedades/</t>
         </is>
       </c>
       <c r="E269" s="3" t="inlineStr">
         <is>
-          <t>HTTP 403 para ambos</t>
+          <t>HTTP 403</t>
         </is>
       </c>
       <c r="F269" s="3" t="inlineStr">
         <is>
-          <t>Gerente: HTTP 403; Vendedor: HTTP 403</t>
+          <t>HTTP 403</t>
         </is>
       </c>
       <c r="G269" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: PreNominaIntegracionViewTest.test_detalle_restringido</t>
+          <t>Prueba automatizada: NovedadesViewTest.test_novedades_restringe_vendedor</t>
         </is>
       </c>
       <c r="H269" s="3" t="inlineStr">
@@ -11790,27 +11790,27 @@
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>Validar que un usuario sin sesión sea enviado al inicio de sesión.</t>
+          <t>Validar que solo el Auxiliar pueda abrir el detalle de la pre-nómina.</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
         <is>
-          <t>Visitante anónimo abre /nomina/reportes/</t>
+          <t>Gerente y Vendedor abren el detalle</t>
         </is>
       </c>
       <c r="E270" s="2" t="inlineStr">
         <is>
-          <t>HTTP 302 a /login/</t>
+          <t>HTTP 403 para ambos</t>
         </is>
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>HTTP 302; redirección a /login/?next=/reportes/nomina/</t>
+          <t>Gerente: HTTP 403; Vendedor: HTTP 403</t>
         </is>
       </c>
       <c r="G270" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ReporteMensualViewTest.test_anonimo_redirige_login</t>
+          <t>Prueba automatizada: PreNominaIntegracionViewTest.test_detalle_restringido</t>
         </is>
       </c>
       <c r="H270" s="2" t="inlineStr">
@@ -11832,27 +11832,27 @@
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>Validar que el Auxiliar Administrativo pueda ver los reportes.</t>
+          <t>Validar que un usuario sin sesión sea enviado al inicio de sesión.</t>
         </is>
       </c>
       <c r="D271" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar abre /nomina/reportes/</t>
+          <t>Visitante anónimo abre /nomina/reportes/</t>
         </is>
       </c>
       <c r="E271" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>HTTP 302 a /login/</t>
         </is>
       </c>
       <c r="F271" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>HTTP 302; redirección a /login/?next=/reportes/nomina/</t>
         </is>
       </c>
       <c r="G271" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ReporteMensualViewTest.test_auxiliar_ve_reportes</t>
+          <t>Prueba automatizada: ReporteMensualViewTest.test_anonimo_redirige_login</t>
         </is>
       </c>
       <c r="H271" s="3" t="inlineStr">
@@ -11874,12 +11874,12 @@
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>Validar que el Gerente pueda ver los reportes de nómina.</t>
+          <t>Validar que el Auxiliar Administrativo pueda ver los reportes.</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
         <is>
-          <t>Gerente abre /nomina/reportes/</t>
+          <t>Auxiliar abre /nomina/reportes/</t>
         </is>
       </c>
       <c r="E272" s="2" t="inlineStr">
@@ -11894,7 +11894,7 @@
       </c>
       <c r="G272" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ReporteMensualViewTest.test_gerente_ve_reportes</t>
+          <t>Prueba automatizada: ReporteMensualViewTest.test_auxiliar_ve_reportes</t>
         </is>
       </c>
       <c r="H272" s="2" t="inlineStr">
@@ -11916,27 +11916,27 @@
       </c>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>Validar que un Vendedor no pueda ver los reportes.</t>
+          <t>Validar que el Gerente pueda ver los reportes de nómina.</t>
         </is>
       </c>
       <c r="D273" s="3" t="inlineStr">
         <is>
-          <t>Vendedor abre /nomina/reportes/</t>
+          <t>Gerente abre /nomina/reportes/</t>
         </is>
       </c>
       <c r="E273" s="3" t="inlineStr">
         <is>
-          <t>HTTP 403</t>
+          <t>HTTP 200</t>
         </is>
       </c>
       <c r="F273" s="3" t="inlineStr">
         <is>
-          <t>HTTP 403</t>
+          <t>HTTP 200</t>
         </is>
       </c>
       <c r="G273" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ReporteMensualViewTest.test_vendedor_no_ve_reportes</t>
+          <t>Prueba automatizada: ReporteMensualViewTest.test_gerente_ve_reportes</t>
         </is>
       </c>
       <c r="H273" s="3" t="inlineStr">
@@ -11958,27 +11958,27 @@
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>Validar que un visitante sin sesión no pueda descargar el PDF.</t>
+          <t>Validar que un Vendedor no pueda ver los reportes.</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
         <is>
-          <t>Anónimo solicita el PDF de 2026-09</t>
+          <t>Vendedor abre /nomina/reportes/</t>
         </is>
       </c>
       <c r="E274" s="2" t="inlineStr">
         <is>
-          <t>HTTP 302 (al inicio de sesión)</t>
+          <t>HTTP 403</t>
         </is>
       </c>
       <c r="F274" s="2" t="inlineStr">
         <is>
-          <t>HTTP 302</t>
+          <t>HTTP 403</t>
         </is>
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ReportePDFViewTest.test_anonimo_no_descarga_pdf</t>
+          <t>Prueba automatizada: ReporteMensualViewTest.test_vendedor_no_ve_reportes</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -12000,27 +12000,27 @@
       </c>
       <c r="C275" s="3" t="inlineStr">
         <is>
-          <t>Validar que un Vendedor no pueda descargar el PDF.</t>
+          <t>Validar que un visitante sin sesión no pueda descargar el PDF.</t>
         </is>
       </c>
       <c r="D275" s="3" t="inlineStr">
         <is>
-          <t>Vendedor solicita el PDF de 2026-09</t>
+          <t>Anónimo solicita el PDF de 2026-09</t>
         </is>
       </c>
       <c r="E275" s="3" t="inlineStr">
         <is>
-          <t>HTTP 403</t>
+          <t>HTTP 302 (al inicio de sesión)</t>
         </is>
       </c>
       <c r="F275" s="3" t="inlineStr">
         <is>
-          <t>HTTP 403</t>
+          <t>HTTP 302</t>
         </is>
       </c>
       <c r="G275" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ReportePDFViewTest.test_vendedor_no_descarga_pdf</t>
+          <t>Prueba automatizada: ReportePDFViewTest.test_anonimo_no_descarga_pdf</t>
         </is>
       </c>
       <c r="H275" s="3" t="inlineStr">
@@ -12037,32 +12037,32 @@
       </c>
       <c r="B276" s="2" t="inlineStr">
         <is>
-          <t>RNF-004</t>
+          <t>RNF-003</t>
         </is>
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>Validar que la nueva contraseña tenga mínimo 8 caracteres.</t>
+          <t>Validar que un Vendedor no pueda descargar el PDF.</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
         <is>
-          <t>nueva: 'Clave12' (7 caracteres)</t>
+          <t>Vendedor solicita el PDF de 2026-09</t>
         </is>
       </c>
       <c r="E276" s="2" t="inlineStr">
         <is>
-          <t>La contraseña debe tener al menos 8 caracteres.</t>
+          <t>HTTP 403</t>
         </is>
       </c>
       <c r="F276" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; mensaje visible: True</t>
+          <t>HTTP 403</t>
         </is>
       </c>
       <c r="G276" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: CambioContrasenaT61Test.test_nueva_contrasena_de_siete_caracteres_muestra_mensaje</t>
+          <t>Prueba automatizada: ReportePDFViewTest.test_vendedor_no_descarga_pdf</t>
         </is>
       </c>
       <c r="H276" s="2" t="inlineStr">
@@ -12084,17 +12084,17 @@
       </c>
       <c r="C277" s="3" t="inlineStr">
         <is>
-          <t>Validar que la nueva contraseña exija una mayúscula.</t>
+          <t>Validar que la nueva contraseña tenga mínimo 8 caracteres.</t>
         </is>
       </c>
       <c r="D277" s="3" t="inlineStr">
         <is>
-          <t>nueva: 'clavesegura2'</t>
+          <t>nueva: 'Clave12' (7 caracteres)</t>
         </is>
       </c>
       <c r="E277" s="3" t="inlineStr">
         <is>
-          <t>La contraseña debe contener al menos una letra mayúscula.</t>
+          <t>La contraseña debe tener al menos 8 caracteres.</t>
         </is>
       </c>
       <c r="F277" s="3" t="inlineStr">
@@ -12104,7 +12104,7 @@
       </c>
       <c r="G277" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: CambioContrasenaT61Test.test_nueva_contrasena_sin_mayuscula_muestra_mensaje</t>
+          <t>Prueba automatizada: CambioContrasenaT61Test.test_nueva_contrasena_de_siete_caracteres_muestra_mensaje</t>
         </is>
       </c>
       <c r="H277" s="3" t="inlineStr">
@@ -12126,17 +12126,17 @@
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>Validar que la nueva contraseña exija una minúscula.</t>
+          <t>Validar que la nueva contraseña exija una mayúscula.</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
         <is>
-          <t>nueva: 'CLAVESEGURA2'</t>
+          <t>nueva: 'clavesegura2'</t>
         </is>
       </c>
       <c r="E278" s="2" t="inlineStr">
         <is>
-          <t>La contraseña debe contener al menos una letra minúscula.</t>
+          <t>La contraseña debe contener al menos una letra mayúscula.</t>
         </is>
       </c>
       <c r="F278" s="2" t="inlineStr">
@@ -12146,7 +12146,7 @@
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: CambioContrasenaT61Test.test_nueva_contrasena_sin_minuscula_muestra_mensaje</t>
+          <t>Prueba automatizada: CambioContrasenaT61Test.test_nueva_contrasena_sin_mayuscula_muestra_mensaje</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr">
@@ -12168,17 +12168,17 @@
       </c>
       <c r="C279" s="3" t="inlineStr">
         <is>
-          <t>Validar que la nueva contraseña exija un número.</t>
+          <t>Validar que la nueva contraseña exija una minúscula.</t>
         </is>
       </c>
       <c r="D279" s="3" t="inlineStr">
         <is>
-          <t>nueva: 'ClaveSegura'</t>
+          <t>nueva: 'CLAVESEGURA2'</t>
         </is>
       </c>
       <c r="E279" s="3" t="inlineStr">
         <is>
-          <t>La contraseña debe contener al menos un número.</t>
+          <t>La contraseña debe contener al menos una letra minúscula.</t>
         </is>
       </c>
       <c r="F279" s="3" t="inlineStr">
@@ -12188,7 +12188,7 @@
       </c>
       <c r="G279" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: CambioContrasenaT61Test.test_nueva_contrasena_sin_numero_muestra_mensaje</t>
+          <t>Prueba automatizada: CambioContrasenaT61Test.test_nueva_contrasena_sin_minuscula_muestra_mensaje</t>
         </is>
       </c>
       <c r="H279" s="3" t="inlineStr">
@@ -12210,27 +12210,27 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>Validar que el validador entregue ayuda.</t>
+          <t>Validar que la nueva contraseña exija un número.</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
         <is>
-          <t>solicitud de texto de ayuda</t>
+          <t>nueva: 'ClaveSegura'</t>
         </is>
       </c>
       <c r="E280" s="2" t="inlineStr">
         <is>
-          <t>El texto de ayuda no está vacío.</t>
+          <t>La contraseña debe contener al menos un número.</t>
         </is>
       </c>
       <c r="F280" s="2" t="inlineStr">
         <is>
-          <t>Texto de ayuda: Mínimo 8 caracteres con mayúsculas, minúsculas y números.</t>
+          <t>HTTP 200; mensaje visible: True</t>
         </is>
       </c>
       <c r="G280" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ComplejidadContrasenaCasosTest.test_contrasena_ayuda</t>
+          <t>Prueba automatizada: CambioContrasenaT61Test.test_nueva_contrasena_sin_numero_muestra_mensaje</t>
         </is>
       </c>
       <c r="H280" s="2" t="inlineStr">
@@ -12252,27 +12252,27 @@
       </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
-          <t>Validar aceptación de contraseña compleja.</t>
+          <t>Validar que el validador entregue ayuda.</t>
         </is>
       </c>
       <c r="D281" s="3" t="inlineStr">
         <is>
-          <t>contraseña: 'Clave#2026'</t>
+          <t>solicitud de texto de ayuda</t>
         </is>
       </c>
       <c r="E281" s="3" t="inlineStr">
         <is>
-          <t>El validador no genera error.</t>
+          <t>El texto de ayuda no está vacío.</t>
         </is>
       </c>
       <c r="F281" s="3" t="inlineStr">
         <is>
-          <t>Resultado: None</t>
+          <t>Texto de ayuda: Mínimo 8 caracteres con mayúsculas, minúsculas y números.</t>
         </is>
       </c>
       <c r="G281" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ComplejidadContrasenaCasosTest.test_contrasena_valida</t>
+          <t>Prueba automatizada: ComplejidadContrasenaCasosTest.test_contrasena_ayuda</t>
         </is>
       </c>
       <c r="H281" s="3" t="inlineStr">
@@ -12294,27 +12294,27 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>Validar que la contraseña requiera mayúscula.</t>
+          <t>Validar aceptación de contraseña compleja.</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
         <is>
-          <t>contraseña: 'clave2026'</t>
+          <t>contraseña: 'Clave#2026'</t>
         </is>
       </c>
       <c r="E282" s="2" t="inlineStr">
         <is>
-          <t>Se produce ValidationError.</t>
+          <t>El validador no genera error.</t>
         </is>
       </c>
       <c r="F282" s="2" t="inlineStr">
         <is>
-          <t>Excepción: ValidationError</t>
+          <t>Resultado: None</t>
         </is>
       </c>
       <c r="G282" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ComplejidadContrasenaCasosTest.test_requiere_mayuscula</t>
+          <t>Prueba automatizada: ComplejidadContrasenaCasosTest.test_contrasena_valida</t>
         </is>
       </c>
       <c r="H282" s="2" t="inlineStr">
@@ -12336,12 +12336,12 @@
       </c>
       <c r="C283" s="3" t="inlineStr">
         <is>
-          <t>Validar que la contraseña requiera minúscula.</t>
+          <t>Validar que la contraseña requiera mayúscula.</t>
         </is>
       </c>
       <c r="D283" s="3" t="inlineStr">
         <is>
-          <t>contraseña: 'CLAVE2026'</t>
+          <t>contraseña: 'clave2026'</t>
         </is>
       </c>
       <c r="E283" s="3" t="inlineStr">
@@ -12356,7 +12356,7 @@
       </c>
       <c r="G283" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ComplejidadContrasenaCasosTest.test_requiere_minuscula</t>
+          <t>Prueba automatizada: ComplejidadContrasenaCasosTest.test_requiere_mayuscula</t>
         </is>
       </c>
       <c r="H283" s="3" t="inlineStr">
@@ -12378,12 +12378,12 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>Validar que la contraseña requiera número.</t>
+          <t>Validar que la contraseña requiera minúscula.</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>contraseña: 'ClaveSegura'</t>
+          <t>contraseña: 'CLAVE2026'</t>
         </is>
       </c>
       <c r="E284" s="2" t="inlineStr">
@@ -12398,7 +12398,7 @@
       </c>
       <c r="G284" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ComplejidadContrasenaCasosTest.test_requiere_numero</t>
+          <t>Prueba automatizada: ComplejidadContrasenaCasosTest.test_requiere_minuscula</t>
         </is>
       </c>
       <c r="H284" s="2" t="inlineStr">
@@ -12420,27 +12420,27 @@
       </c>
       <c r="C285" s="3" t="inlineStr">
         <is>
-          <t>Validar rechazo de contraseña sin mayúscula.</t>
+          <t>Validar que la contraseña requiera número.</t>
         </is>
       </c>
       <c r="D285" s="3" t="inlineStr">
         <is>
-          <t>contraseña: 'clavesegura1'</t>
+          <t>contraseña: 'ClaveSegura'</t>
         </is>
       </c>
       <c r="E285" s="3" t="inlineStr">
         <is>
-          <t>Se informa que falta una mayúscula.</t>
+          <t>Se produce ValidationError.</t>
         </is>
       </c>
       <c r="F285" s="3" t="inlineStr">
         <is>
-          <t>Mensaje mostrado: La contraseña debe contener al menos una letra mayúscula.</t>
+          <t>Excepción: ValidationError</t>
         </is>
       </c>
       <c r="G285" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ValidacionesGestionUsuarioTest.test_contrasena_sin_mayuscula</t>
+          <t>Prueba automatizada: ComplejidadContrasenaCasosTest.test_requiere_numero</t>
         </is>
       </c>
       <c r="H285" s="3" t="inlineStr">
@@ -12462,27 +12462,27 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>Validar rechazo de contraseña sin minúscula.</t>
+          <t>Validar rechazo de contraseña sin mayúscula.</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
         <is>
-          <t>contraseña: 'CLAVESEGURA1'</t>
+          <t>contraseña: 'clavesegura1'</t>
         </is>
       </c>
       <c r="E286" s="2" t="inlineStr">
         <is>
-          <t>Se informa que falta una minúscula.</t>
+          <t>Se informa que falta una mayúscula.</t>
         </is>
       </c>
       <c r="F286" s="2" t="inlineStr">
         <is>
-          <t>Mensaje mostrado: La contraseña debe contener al menos una letra minúscula.</t>
+          <t>Mensaje mostrado: La contraseña debe contener al menos una letra mayúscula.</t>
         </is>
       </c>
       <c r="G286" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ValidacionesGestionUsuarioTest.test_contrasena_sin_minuscula</t>
+          <t>Prueba automatizada: ValidacionesGestionUsuarioTest.test_contrasena_sin_mayuscula</t>
         </is>
       </c>
       <c r="H286" s="2" t="inlineStr">
@@ -12504,27 +12504,27 @@
       </c>
       <c r="C287" s="3" t="inlineStr">
         <is>
-          <t>Validar rechazo de contraseña sin número.</t>
+          <t>Validar rechazo de contraseña sin minúscula.</t>
         </is>
       </c>
       <c r="D287" s="3" t="inlineStr">
         <is>
-          <t>contraseña: 'ClaveSegura'</t>
+          <t>contraseña: 'CLAVESEGURA1'</t>
         </is>
       </c>
       <c r="E287" s="3" t="inlineStr">
         <is>
-          <t>Se informa que falta un número.</t>
+          <t>Se informa que falta una minúscula.</t>
         </is>
       </c>
       <c r="F287" s="3" t="inlineStr">
         <is>
-          <t>Mensaje mostrado: La contraseña debe contener al menos un número.</t>
+          <t>Mensaje mostrado: La contraseña debe contener al menos una letra minúscula.</t>
         </is>
       </c>
       <c r="G287" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: ValidacionesGestionUsuarioTest.test_contrasena_sin_numero</t>
+          <t>Prueba automatizada: ValidacionesGestionUsuarioTest.test_contrasena_sin_minuscula</t>
         </is>
       </c>
       <c r="H287" s="3" t="inlineStr">
@@ -12541,32 +12541,32 @@
       </c>
       <c r="B288" s="2" t="inlineStr">
         <is>
-          <t>RNF-005</t>
+          <t>RNF-004</t>
         </is>
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>Validar autenticación en humo de Vercel</t>
+          <t>Validar rechazo de contraseña sin número.</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
         <is>
-          <t>Locust: 5 usuarios concurrentes</t>
+          <t>contraseña: 'ClaveSegura'</t>
         </is>
       </c>
       <c r="E288" s="2" t="inlineStr">
         <is>
-          <t>p95 &lt;= 2.000 ms y 0 errores</t>
+          <t>Se informa que falta un número.</t>
         </is>
       </c>
       <c r="F288" s="2" t="inlineStr">
         <is>
-          <t>p95 140 ms; 0 errores</t>
+          <t>Mensaje mostrado: La contraseña debe contener al menos un número.</t>
         </is>
       </c>
       <c r="G288" s="2" t="inlineStr">
         <is>
-          <t>Prueba de carga: Locust humo Vercel, 5 usuarios</t>
+          <t>Prueba automatizada: ValidacionesGestionUsuarioTest.test_contrasena_sin_numero</t>
         </is>
       </c>
       <c r="H288" s="2" t="inlineStr">
@@ -12588,32 +12588,32 @@
       </c>
       <c r="C289" s="3" t="inlineStr">
         <is>
-          <t>Validar autenticación bajo carga optimizada</t>
+          <t>Validar autenticación en humo de Vercel</t>
         </is>
       </c>
       <c r="D289" s="3" t="inlineStr">
         <is>
-          <t>Locust: 30 usuarios; POST login</t>
+          <t>Locust: 5 usuarios concurrentes</t>
         </is>
       </c>
       <c r="E289" s="3" t="inlineStr">
         <is>
-          <t>p95 &lt;= 2.000 ms</t>
+          <t>p95 &lt;= 2.000 ms y 0 errores</t>
         </is>
       </c>
       <c r="F289" s="3" t="inlineStr">
         <is>
-          <t>p95 2.700 ms</t>
+          <t>p95 140 ms; 0 errores</t>
         </is>
       </c>
       <c r="G289" s="3" t="inlineStr">
         <is>
-          <t>Supera 2 s solo con 30 inicios de sesión simultáneos en el equipo local (hash PBKDF2 por petición). Un inicio de sesión individual tarda menos de 2 s (CP automatizado de RNF-005) y en Vercel el p95 fue 140 ms.; Prueba de carga: Locust optimizada, login, 30 usuarios</t>
+          <t>Prueba de carga: Locust humo Vercel, 5 usuarios</t>
         </is>
       </c>
       <c r="H289" s="3" t="inlineStr">
         <is>
-          <t>Observación</t>
+          <t>Aprobado</t>
         </is>
       </c>
     </row>
@@ -12630,32 +12630,32 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>Validar que un inicio de sesión válido responda en hasta 2 segundos.</t>
+          <t>Validar autenticación bajo carga optimizada</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
         <is>
-          <t>POST login con correo perf@example.com y contraseña ClaveSegura1</t>
+          <t>Locust: 30 usuarios; POST login</t>
         </is>
       </c>
       <c r="E290" s="2" t="inlineStr">
         <is>
-          <t>HTTP 302 en &lt;= 2,00 s</t>
+          <t>p95 &lt;= 2.000 ms</t>
         </is>
       </c>
       <c r="F290" s="2" t="inlineStr">
         <is>
-          <t>HTTP 302; tiempo medido: 1.695 s</t>
+          <t>p95 2.700 ms</t>
         </is>
       </c>
       <c r="G290" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: RendimientoNominaTest.test_login_valido_hasta_2_segundos</t>
+          <t>Supera 2 s solo con 30 inicios de sesión simultáneos en el equipo local (hash PBKDF2 por petición). Un inicio de sesión individual tarda menos de 2 s (CP automatizado de RNF-005) y en Vercel el p95 fue 140 ms.; Prueba de carga: Locust optimizada, login, 30 usuarios</t>
         </is>
       </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observación</t>
         </is>
       </c>
     </row>
@@ -12667,37 +12667,37 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>RNF-006</t>
+          <t>RNF-005</t>
         </is>
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
-          <t>Validar que la pre-nómina de 200 empleados tarde como máximo 60 segundos.</t>
+          <t>Validar que un inicio de sesión válido responda en hasta 2 segundos.</t>
         </is>
       </c>
       <c r="D291" s="3" t="inlineStr">
         <is>
-          <t>200 usuarios activos con salarios variados; período 2026-09</t>
+          <t>POST login con correo perf@example.com y contraseña ClaveSegura1</t>
         </is>
       </c>
       <c r="E291" s="3" t="inlineStr">
         <is>
-          <t>Tiempo &lt;= 60,00 s</t>
+          <t>HTTP 302 en &lt;= 2,00 s</t>
         </is>
       </c>
       <c r="F291" s="3" t="inlineStr">
         <is>
-          <t>Tiempo medido: 69.13 s para 200 empleados</t>
+          <t>HTTP 302; tiempo medido: 1.614 s</t>
         </is>
       </c>
       <c r="G291" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: RendimientoNominaTest.test_generacion_prenomina_200_empleados_hasta_60_segundos</t>
+          <t>Prueba automatizada: RendimientoNominaTest.test_login_valido_hasta_2_segundos</t>
         </is>
       </c>
       <c r="H291" s="3" t="inlineStr">
         <is>
-          <t>No aprobado</t>
+          <t>Aprobado</t>
         </is>
       </c>
     </row>
@@ -12709,37 +12709,37 @@
       </c>
       <c r="B292" s="2" t="inlineStr">
         <is>
-          <t>RNF-007</t>
+          <t>RNF-006</t>
         </is>
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>Validar consultas filtradas bajo carga base (30 usuarios)</t>
+          <t>Validar que la pre-nómina de 200 empleados tarde como máximo 60 segundos.</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
         <is>
-          <t>Locust: 30 usuarios concurrentes</t>
+          <t>200 usuarios activos con salarios variados; período 2026-09</t>
         </is>
       </c>
       <c r="E292" s="2" t="inlineStr">
         <is>
-          <t>p95 &lt;= 3.000 ms y 0 errores</t>
+          <t>Tiempo &lt;= 60,00 s</t>
         </is>
       </c>
       <c r="F292" s="2" t="inlineStr">
         <is>
-          <t>Mediana 3.500 ms; p95 4.200 ms; 0 errores</t>
+          <t>Tiempo medido: 1.43 s para 200 empleados</t>
         </is>
       </c>
       <c r="G292" s="2" t="inlineStr">
         <is>
-          <t>Defecto encontrado: se abría una conexión nueva a Neon en cada petición. Corregido con CONN_MAX_AGE y CONN_HEALTH_CHECKS; el re-test (carga optimizada) cumple.; Prueba de carga: Locust línea base, 30 usuarios</t>
+          <t>Primera ejecución: No aprobado (69,13 s) por 3 consultas por empleado. Defecto corregido: bonificaciones y horas extra se leen en 2 consultas y las nóminas se insertan con bulk_create.; Prueba automatizada: RendimientoNominaTest.test_generacion_prenomina_200_empleados_hasta_60_segundos</t>
         </is>
       </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
-          <t>No aprobado</t>
+          <t>Aprobado</t>
         </is>
       </c>
     </row>
@@ -12756,7 +12756,7 @@
       </c>
       <c r="C293" s="3" t="inlineStr">
         <is>
-          <t>Validar consultas filtradas bajo carga optimizada</t>
+          <t>Validar consultas filtradas bajo carga base (30 usuarios)</t>
         </is>
       </c>
       <c r="D293" s="3" t="inlineStr">
@@ -12766,22 +12766,22 @@
       </c>
       <c r="E293" s="3" t="inlineStr">
         <is>
-          <t>p95 &lt;= 3.000 ms</t>
+          <t>p95 &lt;= 3.000 ms y 0 errores</t>
         </is>
       </c>
       <c r="F293" s="3" t="inlineStr">
         <is>
-          <t>p95 1.600-1.900 ms; PDF 1.600 ms</t>
+          <t>Mediana 3.500 ms; p95 4.200 ms; 0 errores</t>
         </is>
       </c>
       <c r="G293" s="3" t="inlineStr">
         <is>
-          <t>Re-test tras corregir el defecto de conexiones. Incluye consultas filtradas y exportación PDF.; Prueba de carga: Locust optimizada, consultas, 30 usuarios</t>
+          <t>Defecto encontrado: se abría una conexión nueva a Neon en cada petición. Corregido con CONN_MAX_AGE y CONN_HEALTH_CHECKS; el re-test (carga optimizada) cumple.; Prueba de carga: Locust línea base, 30 usuarios</t>
         </is>
       </c>
       <c r="H293" s="3" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>No aprobado</t>
         </is>
       </c>
     </row>
@@ -12798,27 +12798,27 @@
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>Validar que la auditoría filtrada responda en hasta 3 segundos.</t>
+          <t>Validar consultas filtradas bajo carga optimizada</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
         <is>
-          <t>300 registros de auditoría; filtro de acción CREAR</t>
+          <t>Locust: 30 usuarios concurrentes</t>
         </is>
       </c>
       <c r="E294" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200 en &lt;= 3,00 s</t>
+          <t>p95 &lt;= 3.000 ms</t>
         </is>
       </c>
       <c r="F294" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; tiempo medido: 0.907 s</t>
+          <t>p95 1.600-1.900 ms; PDF 1.600 ms</t>
         </is>
       </c>
       <c r="G294" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: RendimientoNominaTest.test_auditoria_filtrada_hasta_3_segundos</t>
+          <t>Re-test tras corregir el defecto de conexiones. Incluye consultas filtradas y exportación PDF.; Prueba de carga: Locust optimizada, consultas, 30 usuarios</t>
         </is>
       </c>
       <c r="H294" s="2" t="inlineStr">
@@ -12840,12 +12840,12 @@
       </c>
       <c r="C295" s="3" t="inlineStr">
         <is>
-          <t>Validar que el historial filtrado responda en hasta 3 segundos.</t>
+          <t>Validar que la auditoría filtrada responda en hasta 3 segundos.</t>
         </is>
       </c>
       <c r="D295" s="3" t="inlineStr">
         <is>
-          <t>200 usuarios; filtro de período 2026-09</t>
+          <t>300 registros de auditoría; filtro de acción CREAR</t>
         </is>
       </c>
       <c r="E295" s="3" t="inlineStr">
@@ -12855,17 +12855,17 @@
       </c>
       <c r="F295" s="3" t="inlineStr">
         <is>
-          <t>HTTP 403; tiempo medido: 0.674 s</t>
+          <t>HTTP 200; tiempo medido: 0.871 s</t>
         </is>
       </c>
       <c r="G295" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: RendimientoNominaTest.test_historial_filtrado_hasta_3_segundos</t>
+          <t>Prueba automatizada: RendimientoNominaTest.test_auditoria_filtrada_hasta_3_segundos</t>
         </is>
       </c>
       <c r="H295" s="3" t="inlineStr">
         <is>
-          <t>No aprobado</t>
+          <t>Aprobado</t>
         </is>
       </c>
     </row>
@@ -12882,12 +12882,12 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>Validar que la lista filtrada de usuarios responda en hasta 3 segundos.</t>
+          <t>Validar que el historial filtrado responda en hasta 3 segundos.</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
         <is>
-          <t>200 usuarios; filtro nombre=Usuario</t>
+          <t>200 usuarios; empleado con rol Vendedor; filtro de período 2026-09</t>
         </is>
       </c>
       <c r="E296" s="2" t="inlineStr">
@@ -12897,17 +12897,17 @@
       </c>
       <c r="F296" s="2" t="inlineStr">
         <is>
-          <t>HTTP 200; tiempo medido: 23.028 s</t>
+          <t>HTTP 200; tiempo medido: 0.760 s</t>
         </is>
       </c>
       <c r="G296" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: RendimientoNominaTest.test_lista_usuarios_filtrada_hasta_3_segundos</t>
+          <t>Primera ejecución: HTTP 403 por un error de la prueba (el empleado no tenía rol). Se corrigió la prueba.; Prueba automatizada: RendimientoNominaTest.test_historial_filtrado_hasta_3_segundos</t>
         </is>
       </c>
       <c r="H296" s="2" t="inlineStr">
         <is>
-          <t>No aprobado</t>
+          <t>Aprobado</t>
         </is>
       </c>
     </row>
@@ -12919,32 +12919,32 @@
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>RNF-009</t>
+          <t>RNF-007</t>
         </is>
       </c>
       <c r="C297" s="3" t="inlineStr">
         <is>
-          <t>Validar que el error de horas extra conserve el mensaje recibido.</t>
+          <t>Validar que la lista filtrada de usuarios responda en hasta 3 segundos.</t>
         </is>
       </c>
       <c r="D297" s="3" t="inlineStr">
         <is>
-          <t>HoraExtraInvalidaError('hora inválida')</t>
+          <t>200 usuarios; filtro nombre=Usuario</t>
         </is>
       </c>
       <c r="E297" s="3" t="inlineStr">
         <is>
-          <t>Mensaje 'hora inválida'</t>
+          <t>HTTP 200 en &lt;= 3,00 s</t>
         </is>
       </c>
       <c r="F297" s="3" t="inlineStr">
         <is>
-          <t>Mensaje: hora inválida</t>
+          <t>HTTP 200; tiempo medido: 1.224 s</t>
         </is>
       </c>
       <c r="G297" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: MensajesExcepcionesTest.test_mensaje_hora_extra_invalida</t>
+          <t>Primera ejecución: No aprobado (23,03 s) porque cada fila consultaba sus roles (N+1). Defecto corregido: obtener_rol usa los grupos precargados.; Prueba automatizada: RendimientoNominaTest.test_lista_usuarios_filtrada_hasta_3_segundos</t>
         </is>
       </c>
       <c r="H297" s="3" t="inlineStr">
@@ -12966,27 +12966,27 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>Validar que el mensaje de rechazo sin motivo lo indique claramente.</t>
+          <t>Validar que el error de horas extra conserve el mensaje recibido.</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
         <is>
-          <t>MotivoRechazoRequeridoError()</t>
+          <t>HoraExtraInvalidaError('hora inválida')</t>
         </is>
       </c>
       <c r="E298" s="2" t="inlineStr">
         <is>
-          <t>Mensaje con la palabra 'motivo'</t>
+          <t>Mensaje 'hora inválida'</t>
         </is>
       </c>
       <c r="F298" s="2" t="inlineStr">
         <is>
-          <t>Mensaje: Debes escribir el motivo del rechazo de la pre-nómina.</t>
+          <t>Mensaje: hora inválida</t>
         </is>
       </c>
       <c r="G298" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: MensajesExcepcionesTest.test_mensaje_motivo_requerido</t>
+          <t>Prueba automatizada: MensajesExcepcionesTest.test_mensaje_hora_extra_invalida</t>
         </is>
       </c>
       <c r="H298" s="2" t="inlineStr">
@@ -13008,27 +13008,27 @@
       </c>
       <c r="C299" s="3" t="inlineStr">
         <is>
-          <t>Validar que el mensaje de nómina ya calculada incluya el periodo y su estado.</t>
+          <t>Validar que el mensaje de rechazo sin motivo lo indique claramente.</t>
         </is>
       </c>
       <c r="D299" s="3" t="inlineStr">
         <is>
-          <t>NominaYaCalculadaError('2026-09', 'aceptada')</t>
+          <t>MotivoRechazoRequeridoError()</t>
         </is>
       </c>
       <c r="E299" s="3" t="inlineStr">
         <is>
-          <t>Mensaje con '2026-09' y 'aceptada'</t>
+          <t>Mensaje con la palabra 'motivo'</t>
         </is>
       </c>
       <c r="F299" s="3" t="inlineStr">
         <is>
-          <t>Mensaje: La nómina de 2026-09 ya fue calculada y está aceptada. Solo se puede recalcular si el Auxiliar Administrativo la rechaza.</t>
+          <t>Mensaje: Debes escribir el motivo del rechazo de la pre-nómina.</t>
         </is>
       </c>
       <c r="G299" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: MensajesExcepcionesTest.test_mensaje_nomina_ya_calculada</t>
+          <t>Prueba automatizada: MensajesExcepcionesTest.test_mensaje_motivo_requerido</t>
         </is>
       </c>
       <c r="H299" s="3" t="inlineStr">
@@ -13050,27 +13050,27 @@
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>Validar que el mensaje de pre-nómina no pendiente incluya su estado.</t>
+          <t>Validar que el mensaje de nómina ya calculada incluya el periodo y su estado.</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
         <is>
-          <t>PreNominaNoPendienteError('aceptada')</t>
+          <t>NominaYaCalculadaError('2026-09', 'aceptada')</t>
         </is>
       </c>
       <c r="E300" s="2" t="inlineStr">
         <is>
-          <t>Mensaje con 'aceptada'</t>
+          <t>Mensaje con '2026-09' y 'aceptada'</t>
         </is>
       </c>
       <c r="F300" s="2" t="inlineStr">
         <is>
-          <t>Mensaje: Esta pre-nómina ya fue aceptada; no se puede volver a procesar.</t>
+          <t>Mensaje: La nómina de 2026-09 ya fue calculada y está aceptada. Solo se puede recalcular si el Auxiliar Administrativo la rechaza.</t>
         </is>
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: MensajesExcepcionesTest.test_mensaje_prenomina_no_pendiente</t>
+          <t>Prueba automatizada: MensajesExcepcionesTest.test_mensaje_nomina_ya_calculada</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -13092,27 +13092,27 @@
       </c>
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>Validar que el mensaje sin empleados activos incluya el periodo.</t>
+          <t>Validar que el mensaje de pre-nómina no pendiente incluya su estado.</t>
         </is>
       </c>
       <c r="D301" s="3" t="inlineStr">
         <is>
-          <t>SinEmpleadosActivosError('2026-09')</t>
+          <t>PreNominaNoPendienteError('aceptada')</t>
         </is>
       </c>
       <c r="E301" s="3" t="inlineStr">
         <is>
-          <t>Mensaje con '2026-09'</t>
+          <t>Mensaje con 'aceptada'</t>
         </is>
       </c>
       <c r="F301" s="3" t="inlineStr">
         <is>
-          <t>Mensaje: No hay empleados activos para calcular la nómina de 2026-09.</t>
+          <t>Mensaje: Esta pre-nómina ya fue aceptada; no se puede volver a procesar.</t>
         </is>
       </c>
       <c r="G301" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: MensajesExcepcionesTest.test_mensaje_sin_empleados</t>
+          <t>Prueba automatizada: MensajesExcepcionesTest.test_mensaje_prenomina_no_pendiente</t>
         </is>
       </c>
       <c r="H301" s="3" t="inlineStr">
@@ -13129,32 +13129,32 @@
       </c>
       <c r="B302" s="2" t="inlineStr">
         <is>
-          <t>RNF-011</t>
+          <t>RNF-009</t>
         </is>
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>Validar rollback si falla el cálculo de un empleado durante la pre-nómina.</t>
+          <t>Validar que el mensaje sin empleados activos incluya el periodo.</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
         <is>
-          <t>3 empleados activos; calcular_nomina falla en el tercero</t>
+          <t>SinEmpleadosActivosError('2026-09')</t>
         </is>
       </c>
       <c r="E302" s="2" t="inlineStr">
         <is>
-          <t>No quedan nóminas ni solicitud del período</t>
+          <t>Mensaje con '2026-09'</t>
         </is>
       </c>
       <c r="F302" s="2" t="inlineStr">
         <is>
-          <t>Nóminas restantes: 0; solicitudes restantes: 0</t>
+          <t>Mensaje: No hay empleados activos para calcular la nómina de 2026-09.</t>
         </is>
       </c>
       <c r="G302" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: RendimientoNominaTest.test_generar_prenomina_revierte_todo_ante_error_intermedio</t>
+          <t>Prueba automatizada: MensajesExcepcionesTest.test_mensaje_sin_empleados</t>
         </is>
       </c>
       <c r="H302" s="2" t="inlineStr">
@@ -13171,37 +13171,37 @@
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>RNF-016</t>
+          <t>RNF-011</t>
         </is>
       </c>
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>Validar volumen y degradación hasta 200 usuarios</t>
+          <t>Validar rollback si falla el cálculo de un empleado durante la pre-nómina.</t>
         </is>
       </c>
       <c r="D303" s="3" t="inlineStr">
         <is>
-          <t>Locust: entre 20 y 200 usuarios</t>
+          <t>200 empleados activos; el cálculo falla en el tercer empleado</t>
         </is>
       </c>
       <c r="E303" s="3" t="inlineStr">
         <is>
-          <t>Soportar 200 usuarios sin errores</t>
+          <t>No quedan nóminas ni solicitud del período</t>
         </is>
       </c>
       <c r="F303" s="3" t="inlineStr">
         <is>
-          <t>0 errores en 3.546 peticiones; quiebre por latencia aproximadamente a 60 usuarios; throughput aproximado 8,4 req/s</t>
+          <t>Nóminas restantes: 0; solicitudes restantes: 0</t>
         </is>
       </c>
       <c r="G303" s="3" t="inlineStr">
         <is>
-          <t>Soporta 200 usuarios sin errores; los tiempos se degradan desde unos 60 usuarios simultáneos (capacidad cómoda: unos 35).; Prueba de carga: Locust estrés, 20-200 usuarios</t>
+          <t>Prueba automatizada: RendimientoNominaTest.test_generar_prenomina_revierte_todo_ante_error_intermedio</t>
         </is>
       </c>
       <c r="H303" s="3" t="inlineStr">
         <is>
-          <t>Observación</t>
+          <t>Aprobado</t>
         </is>
       </c>
     </row>
@@ -13218,32 +13218,32 @@
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>Validar que la demostración deje al menos 10 registros en cada tabla.</t>
+          <t>Validar volumen y degradación hasta 200 usuarios</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
         <is>
-          <t>poblar_datos_demo --confirmar</t>
+          <t>Locust: entre 20 y 200 usuarios</t>
         </is>
       </c>
       <c r="E304" s="2" t="inlineStr">
         <is>
-          <t>Bonificaciones, horas extra, solicitudes, nóminas y auditoría ≥ 10</t>
+          <t>Soportar 200 usuarios sin errores</t>
         </is>
       </c>
       <c r="F304" s="2" t="inlineStr">
         <is>
-          <t>Registros por tabla: {'bonificaciones': 10, 'horas_extra': 28, 'solicitudes': 26, 'nominas': 106, 'auditoria': 44}</t>
+          <t>0 errores en 3.546 peticiones; quiebre por latencia aproximadamente a 60 usuarios; throughput aproximado 8,4 req/s</t>
         </is>
       </c>
       <c r="G304" s="2" t="inlineStr">
         <is>
-          <t>Prueba automatizada: PoblarDatosDemoTest.test_volumen_por_tabla</t>
+          <t>Soporta 200 usuarios sin errores; los tiempos se degradan desde unos 60 usuarios simultáneos (capacidad cómoda: unos 35).; Prueba de carga: Locust estrés, 20-200 usuarios</t>
         </is>
       </c>
       <c r="H304" s="2" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observación</t>
         </is>
       </c>
     </row>
@@ -13260,27 +13260,27 @@
       </c>
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>Validar que los datos de carga solo se siembren en una base terminada en "carga".</t>
+          <t>Validar que la demostración deje al menos 10 registros en cada tabla.</t>
         </is>
       </c>
       <c r="D305" s="3" t="inlineStr">
         <is>
-          <t>sembrar_datos_carga --confirmar sobre la base de pruebas</t>
+          <t>poblar_datos_demo --confirmar</t>
         </is>
       </c>
       <c r="E305" s="3" t="inlineStr">
         <is>
-          <t>Este comando solo puede ejecutarse sobre una base de datos de carga (nombre terminado en "carga"). Base actual: &lt;nombre&gt;.</t>
+          <t>Bonificaciones, horas extra, solicitudes, nóminas y auditoría ≥ 10</t>
         </is>
       </c>
       <c r="F305" s="3" t="inlineStr">
         <is>
-          <t>Mensaje: Este comando solo puede ejecutarse sobre una base de datos de carga (nombre terminado en "carga"). Base actual: test_neondb.</t>
+          <t>Registros por tabla: {'bonificaciones': 10, 'horas_extra': 28, 'solicitudes': 26, 'nominas': 106, 'auditoria': 44}</t>
         </is>
       </c>
       <c r="G305" s="3" t="inlineStr">
         <is>
-          <t>Prueba automatizada: SembrarDatosCargaTest.test_rechaza_base_de_pruebas</t>
+          <t>Prueba automatizada: PoblarDatosDemoTest.test_volumen_por_tabla</t>
         </is>
       </c>
       <c r="H305" s="3" t="inlineStr">
@@ -13302,38 +13302,80 @@
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
+          <t>Validar que los datos de carga solo se siembren en una base terminada en "carga".</t>
+        </is>
+      </c>
+      <c r="D306" s="2" t="inlineStr">
+        <is>
+          <t>sembrar_datos_carga --confirmar sobre la base de pruebas</t>
+        </is>
+      </c>
+      <c r="E306" s="2" t="inlineStr">
+        <is>
+          <t>Este comando solo puede ejecutarse sobre una base de datos de carga (nombre terminado en "carga"). Base actual: &lt;nombre&gt;.</t>
+        </is>
+      </c>
+      <c r="F306" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje: Este comando solo puede ejecutarse sobre una base de datos de carga (nombre terminado en "carga"). Base actual: test_neondb.</t>
+        </is>
+      </c>
+      <c r="G306" s="2" t="inlineStr">
+        <is>
+          <t>Prueba automatizada: SembrarDatosCargaTest.test_rechaza_base_de_pruebas</t>
+        </is>
+      </c>
+      <c r="H306" s="2" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="3" t="inlineStr">
+        <is>
+          <t>CP306</t>
+        </is>
+      </c>
+      <c r="B307" s="3" t="inlineStr">
+        <is>
+          <t>RNF-016</t>
+        </is>
+      </c>
+      <c r="C307" s="3" t="inlineStr">
+        <is>
           <t>Validar que el sembrado de datos de carga exija confirmación explícita.</t>
         </is>
       </c>
-      <c r="D306" s="2" t="inlineStr">
+      <c r="D307" s="3" t="inlineStr">
         <is>
           <t>sembrar_datos_carga sin --confirmar</t>
         </is>
       </c>
-      <c r="E306" s="2" t="inlineStr">
+      <c r="E307" s="3" t="inlineStr">
         <is>
           <t>Agrega --confirmar para sembrar datos de carga.</t>
         </is>
       </c>
-      <c r="F306" s="2" t="inlineStr">
+      <c r="F307" s="3" t="inlineStr">
         <is>
           <t>Mensaje: Agrega --confirmar para sembrar datos de carga.</t>
         </is>
       </c>
-      <c r="G306" s="2" t="inlineStr">
+      <c r="G307" s="3" t="inlineStr">
         <is>
           <t>Prueba automatizada: SembrarDatosCargaTest.test_requiere_confirmacion</t>
         </is>
       </c>
-      <c r="H306" s="2" t="inlineStr">
+      <c r="H307" s="3" t="inlineStr">
         <is>
           <t>Aprobado</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H306"/>
-  <conditionalFormatting sqref="H2:H306">
+  <autoFilter ref="A1:H307"/>
+  <conditionalFormatting sqref="H2:H307">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>H2="Aprobado"</formula>
     </cfRule>

</xml_diff>